<commit_message>
working on v2.0 docs
</commit_message>
<xml_diff>
--- a/sample_apps/dst_stn_en/dst_knowledge_en.xlsx
+++ b/sample_apps/dst_stn_en/dst_knowledge_en.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nakano\system\dialbb\dialbb-next\sample_apps\dst_stn_en\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1A7D309-7210-419E-B020-03BD0CD79FA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E0499B1-2317-4272-AD2A-601BD4E6106B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{C3566FB2-A815-41D8-9347-99D11DD601B4}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C3566FB2-A815-41D8-9347-99D11DD601B4}"/>
   </bookViews>
   <sheets>
     <sheet name="dialogues" sheetId="2" r:id="rId1"/>

</xml_diff>